<commit_message>
updated with Andy's paths
</commit_message>
<xml_diff>
--- a/Testing_Z-Prime/FLIPR_Analysis_parameters_Run_7_New_Replacement_Options.xlsx
+++ b/Testing_Z-Prime/FLIPR_Analysis_parameters_Run_7_New_Replacement_Options.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danyalepic/Desktop/NIH_VSOAR_2023/aso/Testing_Z-Prime/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pattac/Desktop/aso/Testing_Z-Prime/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF066787-6474-2A4E-ADBD-476428679326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{988F58E8-2BDC-924D-8EB5-851296F468AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1160" windowWidth="28800" windowHeight="11420" xr2:uid="{0CAB9F61-8625-4693-AEA6-DA4D32CF3F2E}"/>
+    <workbookView xWindow="0" yWindow="1160" windowWidth="34080" windowHeight="16720" xr2:uid="{0CAB9F61-8625-4693-AEA6-DA4D32CF3F2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis_Settings" sheetId="2" r:id="rId1"/>
@@ -561,7 +561,7 @@
     <t>Could not measure OR &lt; 2 measurments</t>
   </si>
   <si>
-    <t>/Users/danyalepic/Desktop/NIH_VSOAR_2023/aso/Testing_Z-Prime</t>
+    <t>/Users/pattac/Desktop/aso/Testing_Z-Prime</t>
   </si>
 </sst>
 </file>

</xml_diff>